<commit_message>
added 12/18 rounds to InitialRegression (used for prelim analysis) sheet
</commit_message>
<xml_diff>
--- a/recording_metadata/Cortana_Recording_Metadata.xlsx
+++ b/recording_metadata/Cortana_Recording_Metadata.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="ER" sheetId="1" state="visible" r:id="rId2"/>
@@ -2501,7 +2501,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B35"/>
-  <sheetFormatPr defaultColWidth="12.01953125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.0390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.42"/>
   </cols>
@@ -2773,7 +2773,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q57"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.32"/>
@@ -3946,7 +3946,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="0" t="s">
@@ -4015,7 +4015,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H121"/>
-  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="14.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.92"/>
@@ -6555,7 +6555,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="45.11"/>
   </cols>
@@ -6600,7 +6600,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.23"/>
@@ -7127,7 +7127,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E37"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.53"/>
@@ -7753,7 +7753,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultColWidth="12.01953125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.0390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.86"/>
   </cols>
@@ -7996,7 +7996,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H94"/>
-  <sheetFormatPr defaultColWidth="12.01953125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.0390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="9.59"/>
@@ -9709,7 +9709,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C91"/>
-  <sheetFormatPr defaultColWidth="8.9921875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.86"/>
@@ -10701,7 +10701,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F91"/>
-  <sheetFormatPr defaultColWidth="8.9921875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.42"/>
@@ -12319,8 +12319,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C52"/>
-  <sheetFormatPr defaultColWidth="11.9140625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C55"/>
+  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
@@ -12892,6 +12892,30 @@
       </c>
       <c r="C52" s="0" t="s">
         <v>205</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="57" t="n">
+        <v>45278</v>
+      </c>
+      <c r="B53" s="58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="5" t="n">
+        <v>45278</v>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="54" t="n">
+        <v>45278</v>
+      </c>
+      <c r="B55" s="55" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -12911,7 +12935,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I64"/>
-  <sheetFormatPr defaultColWidth="8.9921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.19"/>
@@ -13583,7 +13607,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E58"/>
-  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.39"/>
@@ -14594,7 +14618,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:S36"/>
-  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.859375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.1"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.11"/>

</xml_diff>